<commit_message>
stablized few issues in Create Map, CreateDS, ValidateImportedValues and ValidateGrpImportValues
</commit_message>
<xml_diff>
--- a/Test Data/Regression/4689052_InHeaderImports/UK_InHeader_ImportTb.xlsx
+++ b/Test Data/Regression/4689052_InHeaderImports/UK_InHeader_ImportTb.xlsx
@@ -23,13 +23,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>2222245_PWE01_1779858394585</t>
-  </si>
-  <si>
-    <t>2222245_PWE02_1779858394585</t>
-  </si>
-  <si>
-    <t>2222245_PWE03_1779858394585</t>
+    <t>2222245_PWE01_1780204192821</t>
+  </si>
+  <si>
+    <t>2222245_PWE02_1780204192821</t>
+  </si>
+  <si>
+    <t>2222245_PWE03_1780204192821</t>
   </si>
   <si>
     <t>Sale of goods, UK</t>

</xml_diff>

<commit_message>
changes done in ENtityGroup and Mapping
</commit_message>
<xml_diff>
--- a/Test Data/Regression/4689052_InHeaderImports/UK_InHeader_ImportTb.xlsx
+++ b/Test Data/Regression/4689052_InHeaderImports/UK_InHeader_ImportTb.xlsx
@@ -23,13 +23,13 @@
     <t>Description</t>
   </si>
   <si>
-    <t>2222245_PWE01_1780204192821</t>
-  </si>
-  <si>
-    <t>2222245_PWE02_1780204192821</t>
-  </si>
-  <si>
-    <t>2222245_PWE03_1780204192821</t>
+    <t>2222245_PWE01_1780424470701</t>
+  </si>
+  <si>
+    <t>2222245_PWE02_1780424470701</t>
+  </si>
+  <si>
+    <t>2222245_PWE03_1780424470701</t>
   </si>
   <si>
     <t>Sale of goods, UK</t>

</xml_diff>